<commit_message>
ME Answer Keys updated
</commit_message>
<xml_diff>
--- a/Data/ME/ME_Quizzes.xlsx
+++ b/Data/ME/ME_Quizzes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\mba\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\mba\Data\ME\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9DCCB6-864F-4592-B8E5-12728E1D8807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EBC860-9993-455B-95A4-CEBC894CD4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="7" xr2:uid="{BD6B024A-9EF8-4B6F-A71B-68FBFE3127E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BD6B024A-9EF8-4B6F-A71B-68FBFE3127E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="1137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="1142">
   <si>
     <t>Some unit</t>
   </si>
@@ -3458,6 +3458,21 @@
   </si>
   <si>
     <t>In national income accounting, the acronym “NI” stands for:</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -3581,7 +3596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -3595,6 +3610,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3930,14 +3948,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6BBF58-BE16-4ADA-8970-1CEE421CBC35}">
   <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="81.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -3956,8 +3974,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -3976,8 +3997,11 @@
       <c r="F2" s="4" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -3996,8 +4020,11 @@
       <c r="F3" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -4016,8 +4043,11 @@
       <c r="F4" s="7" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -4036,8 +4066,11 @@
       <c r="F5" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -4056,8 +4089,11 @@
       <c r="F6" s="7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -4076,8 +4112,11 @@
       <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -4096,8 +4135,11 @@
       <c r="F8" s="7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -4116,8 +4158,11 @@
       <c r="F9" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -4136,8 +4181,11 @@
       <c r="F10" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -4156,8 +4204,11 @@
       <c r="F11" s="7" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -4176,8 +4227,11 @@
       <c r="F12" s="4" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -4196,8 +4250,11 @@
       <c r="F13" s="7" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -4216,8 +4273,11 @@
       <c r="F14" s="4" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -4236,8 +4296,11 @@
       <c r="F15" s="7" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -4256,8 +4319,11 @@
       <c r="F16" s="4" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -4276,8 +4342,11 @@
       <c r="F17" s="7" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -4296,8 +4365,11 @@
       <c r="F18" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -4316,8 +4388,11 @@
       <c r="F19" s="7" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -4336,8 +4411,11 @@
       <c r="F20" s="4" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -4355,6 +4433,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>41</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -4365,7 +4446,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C13B80B8-D450-4B06-80D9-3A3BD392FCDD}">
   <sheetPr codeName="Sheet22"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -4376,7 +4457,7 @@
     <col min="6" max="6" width="63.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -4395,8 +4476,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -4415,8 +4499,11 @@
       <c r="F2" s="4" t="s">
         <v>947</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -4435,8 +4522,11 @@
       <c r="F3" s="7" t="s">
         <v>896</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -4455,8 +4545,11 @@
       <c r="F4" s="7" t="s">
         <v>886</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -4475,8 +4568,11 @@
       <c r="F5" s="4" t="s">
         <v>881</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -4495,8 +4591,11 @@
       <c r="F6" s="7" t="s">
         <v>876</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -4515,8 +4614,11 @@
       <c r="F7" s="4" t="s">
         <v>871</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -4535,8 +4637,11 @@
       <c r="F8" s="7" t="s">
         <v>866</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -4555,8 +4660,11 @@
       <c r="F9" s="4" t="s">
         <v>861</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -4575,8 +4683,11 @@
       <c r="F10" s="1" t="s">
         <v>856</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -4595,8 +4706,11 @@
       <c r="F11" s="7" t="s">
         <v>942</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -4615,8 +4729,11 @@
       <c r="F12" s="4" t="s">
         <v>937</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -4635,8 +4752,11 @@
       <c r="F13" s="7" t="s">
         <v>932</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -4655,8 +4775,11 @@
       <c r="F14" s="4" t="s">
         <v>866</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -4675,8 +4798,11 @@
       <c r="F15" s="7" t="s">
         <v>924</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -4695,8 +4821,11 @@
       <c r="F16" s="4" t="s">
         <v>919</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -4715,8 +4844,11 @@
       <c r="F17" s="7" t="s">
         <v>915</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -4735,8 +4867,11 @@
       <c r="F18" s="4" t="s">
         <v>910</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -4755,8 +4890,11 @@
       <c r="F19" s="7" t="s">
         <v>906</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -4775,8 +4913,11 @@
       <c r="F20" s="4" t="s">
         <v>901</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -4794,6 +4935,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>891</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1138</v>
       </c>
     </row>
   </sheetData>
@@ -4804,7 +4948,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F0330E0-4ED3-4C30-A6E3-1DF832B53A51}">
   <sheetPr codeName="Sheet23"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -4815,7 +4959,7 @@
     <col min="6" max="6" width="47.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -4834,8 +4978,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -4854,8 +5001,11 @@
       <c r="F2" s="4" t="s">
         <v>1035</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -4874,8 +5024,11 @@
       <c r="F3" s="7" t="s">
         <v>984</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -4894,8 +5047,11 @@
       <c r="F4" s="7" t="s">
         <v>930</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -4914,8 +5070,11 @@
       <c r="F5" s="4" t="s">
         <v>973</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -4934,8 +5093,11 @@
       <c r="F6" s="7" t="s">
         <v>969</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -4954,8 +5116,11 @@
       <c r="F7" s="4" t="s">
         <v>964</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -4974,8 +5139,11 @@
       <c r="F8" s="7" t="s">
         <v>866</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -4994,8 +5162,11 @@
       <c r="F9" s="4" t="s">
         <v>957</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -5014,8 +5185,11 @@
       <c r="F10" s="1" t="s">
         <v>952</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -5034,8 +5208,11 @@
       <c r="F11" s="7" t="s">
         <v>1030</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -5054,8 +5231,11 @@
       <c r="F12" s="4" t="s">
         <v>1025</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -5074,8 +5254,11 @@
       <c r="F13" s="7" t="s">
         <v>1021</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -5094,8 +5277,11 @@
       <c r="F14" s="4" t="s">
         <v>980</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -5114,8 +5300,11 @@
       <c r="F15" s="7" t="s">
         <v>1013</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -5134,8 +5323,11 @@
       <c r="F16" s="4" t="s">
         <v>1008</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -5154,8 +5346,11 @@
       <c r="F17" s="7" t="s">
         <v>1003</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -5174,8 +5369,11 @@
       <c r="F18" s="4" t="s">
         <v>999</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -5194,8 +5392,11 @@
       <c r="F19" s="7" t="s">
         <v>994</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -5214,8 +5415,11 @@
       <c r="F20" s="4" t="s">
         <v>989</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -5233,6 +5437,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>979</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1139</v>
       </c>
     </row>
   </sheetData>
@@ -5243,7 +5450,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBCD5B5A-4A3C-4BE1-97F1-DDCA57D30FDF}">
   <sheetPr codeName="Sheet24"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -5254,7 +5461,7 @@
     <col min="6" max="6" width="56.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -5273,8 +5480,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -5293,8 +5503,11 @@
       <c r="F2" s="4" t="s">
         <v>1132</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -5313,8 +5526,11 @@
       <c r="F3" s="7" t="s">
         <v>1078</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -5333,8 +5549,11 @@
       <c r="F4" s="7" t="s">
         <v>1069</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -5353,8 +5572,11 @@
       <c r="F5" s="4" t="s">
         <v>1064</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -5373,8 +5595,11 @@
       <c r="F6" s="7" t="s">
         <v>917</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -5393,8 +5618,11 @@
       <c r="F7" s="4" t="s">
         <v>1055</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -5413,8 +5641,11 @@
       <c r="F8" s="7" t="s">
         <v>1050</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -5433,8 +5664,11 @@
       <c r="F9" s="4" t="s">
         <v>1045</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -5453,8 +5687,11 @@
       <c r="F10" s="1" t="s">
         <v>1040</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -5473,8 +5710,11 @@
       <c r="F11" s="7" t="s">
         <v>1127</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -5493,8 +5733,11 @@
       <c r="F12" s="4" t="s">
         <v>1122</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -5513,8 +5756,11 @@
       <c r="F13" s="7" t="s">
         <v>1117</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -5533,8 +5779,11 @@
       <c r="F14" s="4" t="s">
         <v>1112</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -5553,8 +5802,11 @@
       <c r="F15" s="7" t="s">
         <v>1107</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -5573,8 +5825,11 @@
       <c r="F16" s="4" t="s">
         <v>1103</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -5593,8 +5848,11 @@
       <c r="F17" s="7" t="s">
         <v>1098</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -5613,8 +5871,11 @@
       <c r="F18" s="4" t="s">
         <v>1093</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -5633,8 +5894,11 @@
       <c r="F19" s="7" t="s">
         <v>1088</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -5653,8 +5917,11 @@
       <c r="F20" s="4" t="s">
         <v>1083</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -5672,6 +5939,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>1074</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -5682,7 +5952,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A17CEBF-5DE0-4B64-9EF9-1B93FB7898A8}">
   <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -5692,7 +5962,7 @@
     <col min="6" max="6" width="61.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -5711,8 +5981,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -5731,8 +6004,11 @@
       <c r="F2" s="4" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -5751,8 +6027,11 @@
       <c r="F3" s="7" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -5771,8 +6050,11 @@
       <c r="F4" s="7" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -5791,8 +6073,11 @@
       <c r="F5" s="4" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -5811,8 +6096,11 @@
       <c r="F6" s="7" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -5831,8 +6119,11 @@
       <c r="F7" s="4" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -5851,8 +6142,11 @@
       <c r="F8" s="7" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -5871,8 +6165,11 @@
       <c r="F9" s="4" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -5891,8 +6188,11 @@
       <c r="F10" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -5911,8 +6211,11 @@
       <c r="F11" s="7" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -5931,8 +6234,11 @@
       <c r="F12" s="4" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -5951,8 +6257,11 @@
       <c r="F13" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -5971,8 +6280,11 @@
       <c r="F14" s="4" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -5991,8 +6303,11 @@
       <c r="F15" s="7" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -6011,8 +6326,11 @@
       <c r="F16" s="4" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -6031,8 +6349,11 @@
       <c r="F17" s="7" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -6051,8 +6372,11 @@
       <c r="F18" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -6071,8 +6395,11 @@
       <c r="F19" s="7" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -6091,8 +6418,11 @@
       <c r="F20" s="4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -6110,6 +6440,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>158</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1138</v>
       </c>
     </row>
   </sheetData>
@@ -6120,7 +6453,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4BE7F3-34F9-4711-A205-E91B16249627}">
   <sheetPr codeName="Sheet15"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -6129,7 +6462,7 @@
     <col min="5" max="6" width="50" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -6148,8 +6481,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -6168,8 +6504,11 @@
       <c r="F2" s="4" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -6188,8 +6527,11 @@
       <c r="F3" s="7" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -6208,8 +6550,11 @@
       <c r="F4" s="7" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -6228,8 +6573,11 @@
       <c r="F5" s="4" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -6248,8 +6596,11 @@
       <c r="F6" s="7" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -6268,8 +6619,11 @@
       <c r="F7" s="4" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -6288,8 +6642,11 @@
       <c r="F8" s="7" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -6308,8 +6665,11 @@
       <c r="F9" s="4" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -6328,8 +6688,11 @@
       <c r="F10" s="1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -6348,8 +6711,11 @@
       <c r="F11" s="7" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -6368,8 +6734,11 @@
       <c r="F12" s="4" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -6388,8 +6757,11 @@
       <c r="F13" s="7" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -6408,8 +6780,11 @@
       <c r="F14" s="4" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -6428,8 +6803,11 @@
       <c r="F15" s="7" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -6448,8 +6826,11 @@
       <c r="F16" s="4" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -6468,8 +6849,11 @@
       <c r="F17" s="7" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -6488,8 +6872,11 @@
       <c r="F18" s="4" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -6508,8 +6895,11 @@
       <c r="F19" s="7" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -6528,8 +6918,11 @@
       <c r="F20" s="4" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -6547,6 +6940,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>249</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -6557,7 +6953,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{304C3C23-4DEE-4E0A-8247-26736F25218C}">
   <sheetPr codeName="Sheet16"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -6568,7 +6964,7 @@
     <col min="6" max="6" width="49.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -6587,8 +6983,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -6607,8 +7006,11 @@
       <c r="F2" s="4" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -6627,8 +7029,11 @@
       <c r="F3" s="7" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -6647,8 +7052,11 @@
       <c r="F4" s="7" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -6667,8 +7075,11 @@
       <c r="F5" s="4" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -6687,8 +7098,11 @@
       <c r="F6" s="7" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -6707,8 +7121,11 @@
       <c r="F7" s="4" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -6727,8 +7144,11 @@
       <c r="F8" s="7" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -6747,8 +7167,11 @@
       <c r="F9" s="4" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -6767,8 +7190,11 @@
       <c r="F10" s="1" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -6787,8 +7213,11 @@
       <c r="F11" s="7" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -6807,8 +7236,11 @@
       <c r="F12" s="4" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -6827,8 +7259,11 @@
       <c r="F13" s="7" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -6847,8 +7282,11 @@
       <c r="F14" s="4" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -6867,8 +7305,11 @@
       <c r="F15" s="7" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -6887,8 +7328,11 @@
       <c r="F16" s="4" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -6907,8 +7351,11 @@
       <c r="F17" s="7" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -6927,8 +7374,11 @@
       <c r="F18" s="4" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -6947,8 +7397,11 @@
       <c r="F19" s="7" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -6967,8 +7420,11 @@
       <c r="F20" s="4" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -6986,6 +7442,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>339</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1138</v>
       </c>
     </row>
   </sheetData>
@@ -6996,7 +7455,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08378BA6-1BF3-4FD0-9BAE-FB5A2B8CE2EB}">
   <sheetPr codeName="Sheet17"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -7007,7 +7466,7 @@
     <col min="6" max="6" width="64.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -7026,8 +7485,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -7046,8 +7508,11 @@
       <c r="F2" s="4" t="s">
         <v>485</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -7066,8 +7531,11 @@
       <c r="F3" s="7" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -7086,8 +7554,11 @@
       <c r="F4" s="7" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -7106,8 +7577,11 @@
       <c r="F5" s="4" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -7126,8 +7600,11 @@
       <c r="F6" s="7" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -7146,8 +7623,11 @@
       <c r="F7" s="4" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -7166,8 +7646,11 @@
       <c r="F8" s="7" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -7186,8 +7669,11 @@
       <c r="F9" s="4" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -7206,8 +7692,11 @@
       <c r="F10" s="1" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -7226,8 +7715,11 @@
       <c r="F11" s="7" t="s">
         <v>480</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -7246,8 +7738,11 @@
       <c r="F12" s="4" t="s">
         <v>475</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -7266,8 +7761,11 @@
       <c r="F13" s="7" t="s">
         <v>470</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -7286,8 +7784,11 @@
       <c r="F14" s="4" t="s">
         <v>465</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -7306,8 +7807,11 @@
       <c r="F15" s="7" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -7326,8 +7830,11 @@
       <c r="F16" s="4" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -7346,8 +7853,11 @@
       <c r="F17" s="7" t="s">
         <v>451</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -7366,8 +7876,11 @@
       <c r="F18" s="4" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -7386,8 +7899,11 @@
       <c r="F19" s="7" t="s">
         <v>441</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -7406,8 +7922,11 @@
       <c r="F20" s="4" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -7425,6 +7944,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>429</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1139</v>
       </c>
     </row>
   </sheetData>
@@ -7435,7 +7957,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA73C3A8-79CB-40AC-AB75-DB302CD8DE75}">
   <sheetPr codeName="Sheet18"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -7446,7 +7968,7 @@
     <col min="6" max="6" width="45.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -7465,8 +7987,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -7485,8 +8010,11 @@
       <c r="F2" s="4" t="s">
         <v>576</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -7505,8 +8033,11 @@
       <c r="F3" s="7" t="s">
         <v>490</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -7525,8 +8056,11 @@
       <c r="F4" s="7" t="s">
         <v>520</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -7545,8 +8079,11 @@
       <c r="F5" s="4" t="s">
         <v>515</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -7565,8 +8102,11 @@
       <c r="F6" s="7" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -7585,8 +8125,11 @@
       <c r="F7" s="4" t="s">
         <v>505</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -7605,8 +8148,11 @@
       <c r="F8" s="7" t="s">
         <v>500</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -7625,8 +8171,11 @@
       <c r="F9" s="4" t="s">
         <v>495</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -7645,8 +8194,11 @@
       <c r="F10" s="1" t="s">
         <v>490</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -7665,8 +8217,11 @@
       <c r="F11" s="7" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -7685,8 +8240,11 @@
       <c r="F12" s="4" t="s">
         <v>492</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -7705,8 +8263,11 @@
       <c r="F13" s="7" t="s">
         <v>562</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -7725,8 +8286,11 @@
       <c r="F14" s="4" t="s">
         <v>557</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -7745,8 +8309,11 @@
       <c r="F15" s="7" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -7765,8 +8332,11 @@
       <c r="F16" s="4" t="s">
         <v>547</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -7785,8 +8355,11 @@
       <c r="F17" s="7" t="s">
         <v>542</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -7805,8 +8378,11 @@
       <c r="F18" s="4" t="s">
         <v>527</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -7825,8 +8401,11 @@
       <c r="F19" s="7" t="s">
         <v>538</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -7845,8 +8424,11 @@
       <c r="F20" s="4" t="s">
         <v>533</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -7864,6 +8446,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>525</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>
@@ -7874,7 +8459,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30A82CDA-3A77-407D-9B46-2FE4E0A4085B}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -7885,7 +8470,7 @@
     <col min="6" max="6" width="56.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -7904,8 +8489,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -7924,8 +8512,11 @@
       <c r="F2" s="4" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -7944,8 +8535,11 @@
       <c r="F3" s="7" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -7964,8 +8558,11 @@
       <c r="F4" s="7" t="s">
         <v>609</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -7984,8 +8581,11 @@
       <c r="F5" s="4" t="s">
         <v>606</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -8004,8 +8604,11 @@
       <c r="F6" s="7" t="s">
         <v>601</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8024,8 +8627,11 @@
       <c r="F7" s="4" t="s">
         <v>596</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -8044,8 +8650,11 @@
       <c r="F8" s="7" t="s">
         <v>591</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -8064,8 +8673,11 @@
       <c r="F9" s="4" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -8084,8 +8696,11 @@
       <c r="F10" s="1" t="s">
         <v>581</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -8104,8 +8719,11 @@
       <c r="F11" s="7" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -8124,8 +8742,11 @@
       <c r="F12" s="4" t="s">
         <v>664</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -8144,8 +8765,11 @@
       <c r="F13" s="7" t="s">
         <v>659</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -8164,8 +8788,11 @@
       <c r="F14" s="4" t="s">
         <v>654</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -8184,8 +8811,11 @@
       <c r="F15" s="7" t="s">
         <v>649</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -8204,8 +8834,11 @@
       <c r="F16" s="4" t="s">
         <v>644</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -8224,8 +8857,11 @@
       <c r="F17" s="7" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -8244,8 +8880,11 @@
       <c r="F18" s="4" t="s">
         <v>634</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -8264,8 +8903,11 @@
       <c r="F19" s="7" t="s">
         <v>629</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -8284,8 +8926,11 @@
       <c r="F20" s="4" t="s">
         <v>624</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -8303,6 +8948,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>614</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1140</v>
       </c>
     </row>
   </sheetData>
@@ -8313,7 +8961,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081C07D9-C5DF-44D5-BB3B-B4429E3E1AFB}">
   <sheetPr codeName="Sheet20"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -8324,7 +8972,7 @@
     <col min="6" max="6" width="49.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -8343,8 +8991,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -8363,8 +9014,11 @@
       <c r="F2" s="4" t="s">
         <v>704</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -8383,8 +9037,11 @@
       <c r="F3" s="7" t="s">
         <v>717</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -8403,8 +9060,11 @@
       <c r="F4" s="7" t="s">
         <v>707</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -8423,8 +9083,11 @@
       <c r="F5" s="4" t="s">
         <v>702</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -8443,8 +9106,11 @@
       <c r="F6" s="7" t="s">
         <v>697</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8463,8 +9129,11 @@
       <c r="F7" s="4" t="s">
         <v>692</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -8483,8 +9152,11 @@
       <c r="F8" s="7" t="s">
         <v>688</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -8503,8 +9175,11 @@
       <c r="F9" s="4" t="s">
         <v>683</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -8523,8 +9198,11 @@
       <c r="F10" s="1" t="s">
         <v>678</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -8543,8 +9221,11 @@
       <c r="F11" s="7" t="s">
         <v>756</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -8563,8 +9244,11 @@
       <c r="F12" s="4" t="s">
         <v>751</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -8583,8 +9267,11 @@
       <c r="F13" s="7" t="s">
         <v>746</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -8603,8 +9290,11 @@
       <c r="F14" s="4" t="s">
         <v>742</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -8623,8 +9313,11 @@
       <c r="F15" s="7" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -8643,8 +9336,11 @@
       <c r="F16" s="4" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -8663,8 +9359,11 @@
       <c r="F17" s="7" t="s">
         <v>732</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -8683,8 +9382,11 @@
       <c r="F18" s="4" t="s">
         <v>689</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -8703,8 +9405,11 @@
       <c r="F19" s="7" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -8723,8 +9428,11 @@
       <c r="F20" s="4" t="s">
         <v>722</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -8742,6 +9450,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>712</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1140</v>
       </c>
     </row>
   </sheetData>
@@ -8752,7 +9463,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3129BFE8-F168-4325-AAD5-E87A540125E5}">
   <sheetPr codeName="Sheet21"/>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -8763,7 +9474,7 @@
     <col min="6" max="6" width="47.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>122</v>
       </c>
@@ -8782,8 +9493,11 @@
       <c r="F1" s="10" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="13" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>116</v>
       </c>
@@ -8802,8 +9516,11 @@
       <c r="F2" s="4" t="s">
         <v>851</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>52</v>
       </c>
@@ -8822,8 +9539,11 @@
       <c r="F3" s="7" t="s">
         <v>799</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -8842,8 +9562,11 @@
       <c r="F4" s="7" t="s">
         <v>789</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -8862,8 +9585,11 @@
       <c r="F5" s="4" t="s">
         <v>784</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>29</v>
       </c>
@@ -8882,8 +9608,11 @@
       <c r="F6" s="7" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="15" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
@@ -8902,8 +9631,11 @@
       <c r="F7" s="4" t="s">
         <v>775</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>17</v>
       </c>
@@ -8922,8 +9654,11 @@
       <c r="F8" s="7" t="s">
         <v>770</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G8" s="15" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -8942,8 +9677,11 @@
       <c r="F9" s="4" t="s">
         <v>767</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>5</v>
       </c>
@@ -8962,8 +9700,11 @@
       <c r="F10" s="1" t="s">
         <v>762</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G10" s="15" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>110</v>
       </c>
@@ -8982,8 +9723,11 @@
       <c r="F11" s="7" t="s">
         <v>846</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>104</v>
       </c>
@@ -9002,8 +9746,11 @@
       <c r="F12" s="4" t="s">
         <v>434</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -9022,8 +9769,11 @@
       <c r="F13" s="7" t="s">
         <v>839</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>92</v>
       </c>
@@ -9042,8 +9792,11 @@
       <c r="F14" s="4" t="s">
         <v>834</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>86</v>
       </c>
@@ -9062,8 +9815,11 @@
       <c r="F15" s="7" t="s">
         <v>829</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>80</v>
       </c>
@@ -9082,8 +9838,11 @@
       <c r="F16" s="4" t="s">
         <v>824</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -9102,8 +9861,11 @@
       <c r="F17" s="7" t="s">
         <v>819</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>68</v>
       </c>
@@ -9122,8 +9884,11 @@
       <c r="F18" s="4" t="s">
         <v>814</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>64</v>
       </c>
@@ -9142,8 +9907,11 @@
       <c r="F19" s="7" t="s">
         <v>809</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
@@ -9162,8 +9930,11 @@
       <c r="F20" s="4" t="s">
         <v>804</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
@@ -9181,6 +9952,9 @@
       </c>
       <c r="F21" s="4" t="s">
         <v>794</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>1141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>